<commit_message>
Update product codes spreadsheet to reflect recent changes in product data organization
</commit_message>
<xml_diff>
--- a/data/products/codes.xlsx
+++ b/data/products/codes.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D5366E4-61E9-45AC-B63F-580015A5E4ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CE2D4C7-6006-413B-B372-C7C0852FCB87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="838" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2986,7 +2986,7 @@
         <v>1</v>
       </c>
       <c r="B64" s="13">
-        <v>40401001</v>
+        <v>42401001</v>
       </c>
       <c r="C64" s="12" t="s">
         <v>110</v>
@@ -3001,7 +3001,7 @@
         <v>2</v>
       </c>
       <c r="B65" s="13">
-        <v>40401002</v>
+        <v>42401002</v>
       </c>
       <c r="C65" s="12" t="s">
         <v>55</v>
@@ -3016,7 +3016,7 @@
         <v>3</v>
       </c>
       <c r="B66" s="13">
-        <v>40401003</v>
+        <v>42401003</v>
       </c>
       <c r="C66" s="15" t="s">
         <v>56</v>
@@ -3031,7 +3031,7 @@
         <v>4</v>
       </c>
       <c r="B67" s="13">
-        <v>40401004</v>
+        <v>42401004</v>
       </c>
       <c r="C67" s="16" t="s">
         <v>57</v>
@@ -3046,7 +3046,7 @@
         <v>5</v>
       </c>
       <c r="B68" s="13">
-        <v>40401005</v>
+        <v>42401005</v>
       </c>
       <c r="C68" s="16" t="s">
         <v>58</v>
@@ -3061,7 +3061,7 @@
         <v>6</v>
       </c>
       <c r="B69" s="13">
-        <v>40401006</v>
+        <v>42401006</v>
       </c>
       <c r="C69" s="16" t="s">
         <v>59</v>
@@ -3076,7 +3076,7 @@
         <v>7</v>
       </c>
       <c r="B70" s="13">
-        <v>40401007</v>
+        <v>42401007</v>
       </c>
       <c r="C70" s="16" t="s">
         <v>60</v>

</xml_diff>

<commit_message>
Update product dimensions in clean-products.json and refresh codes spreadsheet
- Adjusted dimensions for specific products in clean-products.json to ensure accurate representation.
- Updated the codes spreadsheet to reflect recent changes in product data organization, enhancing consistency across datasets.
</commit_message>
<xml_diff>
--- a/data/products/codes.xlsx
+++ b/data/products/codes.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CE2D4C7-6006-413B-B372-C7C0852FCB87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C69A9EE-4125-4CC5-AA6E-2A23EADD31C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="838" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="193">
   <si>
     <t>موج العاشر من رمضان</t>
   </si>
@@ -776,9 +776,6 @@
   </si>
   <si>
     <t>بان مارى كاونتر سعة 1 حلة GN1/1 (غير شامل الحلل)</t>
-  </si>
-  <si>
-    <t>بوتاجاز 4 شعلة بفرن كبير</t>
   </si>
   <si>
     <t>بوتاجاز أرضى 1 شعلة مصنع من شاسيه زوايا حديد</t>
@@ -1813,7 +1810,7 @@
     </row>
     <row r="4" spans="1:7" ht="20.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="61" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B4" s="61"/>
       <c r="C4" s="61"/>
@@ -1836,7 +1833,7 @@
         <v>8</v>
       </c>
       <c r="B6" s="63" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C6" s="64" t="s">
         <v>1</v>
@@ -1847,7 +1844,7 @@
       <c r="E6" s="64"/>
       <c r="F6" s="65"/>
       <c r="G6" s="63" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="26.45" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1905,7 +1902,7 @@
         <v>40101002</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>165</v>
+        <v>6</v>
       </c>
       <c r="D10" s="13">
         <v>120</v>
@@ -2073,7 +2070,7 @@
         <v>40101010</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D18" s="14">
         <v>40</v>
@@ -2136,7 +2133,7 @@
         <v>40101013</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D21" s="13">
         <v>70</v>
@@ -2157,7 +2154,7 @@
         <v>40101014</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D22" s="14">
         <v>150</v>
@@ -2178,7 +2175,7 @@
         <v>40101015</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D23" s="14">
         <v>180</v>
@@ -2199,7 +2196,7 @@
         <v>40101016</v>
       </c>
       <c r="C24" s="15" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D24" s="14">
         <v>210</v>
@@ -2420,7 +2417,7 @@
         <v>40201010</v>
       </c>
       <c r="C35" s="15" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D35" s="14">
         <v>120</v>
@@ -2894,7 +2891,7 @@
         <v>40401002</v>
       </c>
       <c r="C59" s="16" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D59" s="17">
         <v>80</v>
@@ -2915,7 +2912,7 @@
         <v>40401003</v>
       </c>
       <c r="C60" s="16" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D60" s="17">
         <v>80</v>
@@ -2936,7 +2933,7 @@
         <v>40401004</v>
       </c>
       <c r="C61" s="16" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D61" s="17">
         <v>80</v>
@@ -2957,7 +2954,7 @@
         <v>40401005</v>
       </c>
       <c r="C62" s="16" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D62" s="17">
         <v>80</v>
@@ -3221,7 +3218,7 @@
         <v>40601004</v>
       </c>
       <c r="C78" s="15" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D78" s="13">
         <v>120</v>
@@ -3506,7 +3503,7 @@
         <v>40801002</v>
       </c>
       <c r="C93" s="16" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D93" s="17">
         <v>80</v>
@@ -3816,7 +3813,7 @@
     </row>
     <row r="109" spans="1:7" ht="28.15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A109" s="25" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B109" s="52"/>
       <c r="C109" s="26"/>
@@ -3833,7 +3830,7 @@
         <v>40902001</v>
       </c>
       <c r="C110" s="15" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D110" s="14">
         <v>80</v>
@@ -3854,7 +3851,7 @@
         <v>40902002</v>
       </c>
       <c r="C111" s="16" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D111" s="17">
         <v>80</v>
@@ -3875,7 +3872,7 @@
         <v>40902003</v>
       </c>
       <c r="C112" s="16" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D112" s="17">
         <v>80</v>
@@ -3896,7 +3893,7 @@
         <v>40902004</v>
       </c>
       <c r="C113" s="15" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D113" s="17">
         <v>120</v>
@@ -3917,7 +3914,7 @@
         <v>40902005</v>
       </c>
       <c r="C114" s="16" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D114" s="17">
         <v>120</v>
@@ -4217,7 +4214,7 @@
     </row>
     <row r="130" spans="1:7" ht="28.15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A130" s="25" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B130" s="52"/>
       <c r="C130" s="26"/>
@@ -4318,7 +4315,7 @@
         <v>41002005</v>
       </c>
       <c r="C135" s="31" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D135" s="21">
         <v>150</v>
@@ -4339,7 +4336,7 @@
         <v>41002006</v>
       </c>
       <c r="C136" s="31" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D136" s="21">
         <v>180</v>
@@ -4354,7 +4351,7 @@
     </row>
     <row r="137" spans="1:7" ht="28.15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A137" s="25" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B137" s="52"/>
       <c r="C137" s="26"/>
@@ -4445,7 +4442,7 @@
         <v>41101001</v>
       </c>
       <c r="C142" s="10" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D142" s="20"/>
       <c r="E142" s="20"/>
@@ -4460,7 +4457,7 @@
         <v>41101002</v>
       </c>
       <c r="C143" s="15" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D143" s="21"/>
       <c r="E143" s="21"/>
@@ -4475,7 +4472,7 @@
         <v>41101003</v>
       </c>
       <c r="C144" s="15" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D144" s="21"/>
       <c r="E144" s="21"/>
@@ -4501,7 +4498,7 @@
         <v>41201001</v>
       </c>
       <c r="C146" s="10" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D146" s="11">
         <v>70</v>
@@ -4522,7 +4519,7 @@
         <v>41201002</v>
       </c>
       <c r="C147" s="12" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D147" s="13">
         <v>140</v>
@@ -4537,7 +4534,7 @@
     </row>
     <row r="148" spans="1:7" ht="28.15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A148" s="25" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B148" s="52"/>
       <c r="C148" s="26"/>

</xml_diff>